<commit_message>
datos: añade la cuenta de X del ministro de Hacienda
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -12246,6 +12246,16 @@
           <t>Arcadi España García</t>
         </is>
       </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>ArcadiSD</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="I297" t="inlineStr">
         <is>
           <t>informacion.hacienda@hacienda.gob.es</t>
@@ -12254,6 +12264,11 @@
       <c r="J297" t="inlineStr">
         <is>
           <t>Ministro de Hacienda</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: fechas de actividad en X de las altas de Congreso y Senado
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -31291,6 +31291,11 @@
           <t>BrigidaPachon</t>
         </is>
       </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>2025-09-02</t>
+        </is>
+      </c>
       <c r="I667" t="inlineStr">
         <is>
           <t>brigida.pachon@congreso.es</t>
@@ -31309,6 +31314,11 @@
       <c r="M667" t="inlineStr">
         <is>
           <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="Q667" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -31382,6 +31392,11 @@
           <t>diegotaiboPSOE</t>
         </is>
       </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>2021-06-30</t>
+        </is>
+      </c>
       <c r="I670" t="inlineStr">
         <is>
           <t>diego.taibo@congreso.es</t>
@@ -31400,6 +31415,11 @@
       <c r="M670" t="inlineStr">
         <is>
           <t>Coruña (A)</t>
+        </is>
+      </c>
+      <c r="Q670" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -60184,6 +60204,11 @@
           <t>_angel_pelayo</t>
         </is>
       </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="K1376" t="inlineStr">
         <is>
           <t>Senador/a</t>
@@ -60197,6 +60222,11 @@
       <c r="N1376" t="inlineStr">
         <is>
           <t>Comunidad Autónoma de Extremadura</t>
+        </is>
+      </c>
+      <c r="Q1376" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -60216,6 +60246,11 @@
           <t>rafaguiamarques</t>
         </is>
       </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="K1377" t="inlineStr">
         <is>
           <t>Senador/a</t>
@@ -60229,6 +60264,11 @@
       <c r="N1377" t="inlineStr">
         <is>
           <t>Comunidad Autónoma de Aragón</t>
+        </is>
+      </c>
+      <c r="Q1377" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -60248,6 +60288,11 @@
           <t>Coronelvox</t>
         </is>
       </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="K1378" t="inlineStr">
         <is>
           <t>Senador/a</t>
@@ -60261,6 +60306,11 @@
       <c r="N1378" t="inlineStr">
         <is>
           <t>Comunidad Autónoma de Aragón</t>
+        </is>
+      </c>
+      <c r="Q1378" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -60280,6 +60330,11 @@
           <t>jesusraguirre</t>
         </is>
       </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="K1379" t="inlineStr">
         <is>
           <t>Senador/a</t>
@@ -60293,6 +60348,11 @@
       <c r="N1379" t="inlineStr">
         <is>
           <t>Comunidad Autónoma de Andalucía</t>
+        </is>
+      </c>
+      <c r="Q1379" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -60312,6 +60372,11 @@
           <t>neusmassanet</t>
         </is>
       </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>2025-11-13</t>
+        </is>
+      </c>
       <c r="K1380" t="inlineStr">
         <is>
           <t>Senador/a</t>
@@ -60325,6 +60390,11 @@
       <c r="M1380" t="inlineStr">
         <is>
           <t>Eivissa-Formentera</t>
+        </is>
+      </c>
+      <c r="Q1380" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -60344,6 +60414,11 @@
           <t>mjmonteroc</t>
         </is>
       </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="K1381" t="inlineStr">
         <is>
           <t>Senador/a</t>
@@ -60357,6 +60432,11 @@
       <c r="N1381" t="inlineStr">
         <is>
           <t>Comunidad Autónoma de Andalucía</t>
+        </is>
+      </c>
+      <c r="Q1381" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -60376,6 +60456,11 @@
           <t>oblader</t>
         </is>
       </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="K1382" t="inlineStr">
         <is>
           <t>Senador/a</t>
@@ -60389,6 +60474,11 @@
       <c r="N1382" t="inlineStr">
         <is>
           <t>Comunidad Autónoma de Andalucía</t>
+        </is>
+      </c>
+      <c r="Q1382" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -60462,6 +60552,11 @@
           <t>jmreniu</t>
         </is>
       </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="E1385" t="inlineStr">
         <is>
           <t>jmreniu.bsky.social</t>
@@ -60485,6 +60580,11 @@
       <c r="N1385" t="inlineStr">
         <is>
           <t>Comunidad Autónoma de Cataluña</t>
+        </is>
+      </c>
+      <c r="Q1385" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="S1385" t="inlineStr">
@@ -60519,6 +60619,11 @@
           <t>Alvaro_Zancajo</t>
         </is>
       </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="K1386" t="inlineStr">
         <is>
           <t>Senador/a</t>
@@ -60532,6 +60637,11 @@
       <c r="N1386" t="inlineStr">
         <is>
           <t>Comunidad Autónoma de Andalucía</t>
+        </is>
+      </c>
+      <c r="Q1386" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>

</xml_diff>